<commit_message>
added bin no and bin type in the planned schedule
</commit_message>
<xml_diff>
--- a/template/Planned_Schedule_Template.xlsx
+++ b/template/Planned_Schedule_Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
   <si>
     <t>NO. PENDAFTARAN KENDERAAN</t>
   </si>
@@ -45,6 +45,12 @@
   </si>
   <si>
     <t>END DATE</t>
+  </si>
+  <si>
+    <t>BIN NO</t>
+  </si>
+  <si>
+    <t>BIN TYPE</t>
   </si>
 </sst>
 </file>
@@ -387,7 +393,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J1000"/>
+  <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="true" style="0"/>
@@ -402,7 +408,7 @@
     <col min="10" max="10" width="14" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -433,6 +439,12 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" spans="1:10">
       <c r="I2" s="1"/>

</xml_diff>